<commit_message>
Refresh API and notification QA docs
- update API test case workbooks for community, media, notes, notifications, profile, reading, and session coverage

- add API route pattern guidance for endpoint testing

- move notification test cases and rule documents into a dedicated Notifications folder
</commit_message>
<xml_diff>
--- a/qa-docs/test-cases/API/API_VerseByVerse_Media_Upload_Test_Cases.xlsx
+++ b/qa-docs/test-cases/API/API_VerseByVerse_Media_Upload_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\versebyverse-quality-engineering\qa-docs\test-cases\API\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF38B7A-BB6C-43ED-A84A-ECBAFCADD6B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C902E9F-3356-4786-B3AC-A1DD22204545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28890" yWindow="4035" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -64,9 +64,6 @@
     <t>Functional</t>
   </si>
   <si>
-    <t>Not Run</t>
-  </si>
-  <si>
     <t>Validation</t>
   </si>
   <si>
@@ -242,6 +239,9 @@
   </si>
   <si>
     <t>VerseByVerse - API Media Upload Test Cases</t>
+  </si>
+  <si>
+    <t>Passed</t>
   </si>
 </sst>
 </file>
@@ -636,7 +636,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -686,63 +686,63 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
         <v>28</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
         <v>29</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>30</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
         <v>11</v>
       </c>
       <c r="J3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K3" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>33</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
         <v>34</v>
       </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>35</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>36</v>
-      </c>
-      <c r="H4" t="s">
-        <v>37</v>
       </c>
       <c r="I4" t="s">
         <v>11</v>
@@ -751,103 +751,103 @@
         <v>12</v>
       </c>
       <c r="K4" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
         <v>38</v>
       </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>39</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>40</v>
       </c>
-      <c r="G5" t="s">
-        <v>41</v>
-      </c>
       <c r="H5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K5" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
         <v>42</v>
       </c>
-      <c r="B6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>43</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>44</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>45</v>
       </c>
-      <c r="G6" t="s">
-        <v>46</v>
-      </c>
       <c r="H6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K6" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
         <v>47</v>
       </c>
-      <c r="B7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>48</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>49</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>50</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
         <v>51</v>
-      </c>
-      <c r="G7" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" t="s">
-        <v>52</v>
       </c>
       <c r="I7" t="s">
         <v>11</v>
@@ -856,68 +856,68 @@
         <v>12</v>
       </c>
       <c r="K7" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" t="s">
         <v>53</v>
       </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>54</v>
       </c>
-      <c r="E8" t="s">
-        <v>55</v>
-      </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I8" t="s">
         <v>11</v>
       </c>
       <c r="J8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
         <v>56</v>
       </c>
-      <c r="B9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>57</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" t="s">
         <v>58</v>
       </c>
-      <c r="E9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" t="s">
         <v>59</v>
-      </c>
-      <c r="G9" t="s">
-        <v>23</v>
-      </c>
-      <c r="H9" t="s">
-        <v>60</v>
       </c>
       <c r="I9" t="s">
         <v>11</v>
@@ -926,112 +926,112 @@
         <v>12</v>
       </c>
       <c r="K9" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" t="s">
         <v>61</v>
       </c>
-      <c r="B10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" t="s">
-        <v>62</v>
-      </c>
       <c r="E10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I10" t="s">
         <v>11</v>
       </c>
       <c r="J10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K10" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" t="s">
         <v>63</v>
       </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" t="s">
         <v>24</v>
-      </c>
-      <c r="D11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" t="s">
-        <v>65</v>
-      </c>
-      <c r="F11" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" t="s">
-        <v>25</v>
       </c>
       <c r="I11" t="s">
         <v>11</v>
       </c>
       <c r="J11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K11" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
         <v>66</v>
       </c>
-      <c r="B12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>67</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>68</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>69</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>70</v>
       </c>
-      <c r="G12" t="s">
-        <v>71</v>
-      </c>
       <c r="H12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K12" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1039,6 +1039,11 @@
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K1048576" xr:uid="{3D5A0F38-2C52-4CF1-A4E2-31057EAB5F12}">
+      <formula1>"Passed,Failed,Blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>